<commit_message>
Updated project tracker spreadsheet
</commit_message>
<xml_diff>
--- a/docs/standards/SJTDM_TAZ_Migration_Project_Control.xlsx
+++ b/docs/standards/SJTDM_TAZ_Migration_Project_Control.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kschellinger\SJTPO_Git\SJTDM_TAZ_Migration\docs\standards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E9025B6-D93D-495D-88BB-DF702857C25D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF78DE4B-6FA1-4EA9-B0FB-2AD7A5D2E0DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1500" yWindow="930" windowWidth="29010" windowHeight="14370" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="810" windowWidth="29010" windowHeight="14370" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="336">
   <si>
     <t>SJTDM TAZ Migration and Data Validation – Project Control Workbook</t>
   </si>
@@ -1028,10 +1028,25 @@
     <t>Column5</t>
   </si>
   <si>
-    <t>Core project objective.  First-pass review of recreational model TAZs completed. TAZs containing significant recreational land-use patterns and sub-census-block characteristics identified. Findings indicate that preservation of model-relevant land-use geography is more important than geometric similarity between legacy and proposed TAZ boundaries.</t>
-  </si>
-  <si>
     <t>Recreational model screening methodology tested. Initial review confirms geometry-only comparisons are insufficient for evaluating migration quality. QA/QC framework shall evaluate preservation of socioeconomic and recreational model characteristics in addition to geometric correspondence.</t>
+  </si>
+  <si>
+    <t>Core project objective.  First-pass review of recreational model TAZs completed. A first-pass review of all 534 recreational model TAZs was completed. A total of 169 TAZs (31.6%) were identified as containing significant sub-census-block characteristics and were exported to REC_MODEL_SUB_Y for further evaluation. Impact assessment determined that only 45 TAZs (8.4%) exhibited Moderate or High potential effects on demographic allocation under a pure 2020 Census Block methodology. The remaining 489 TAZs (91.6%) exhibited Low or No Significant impact.</t>
+  </si>
+  <si>
+    <t>DI-009</t>
+  </si>
+  <si>
+    <t>REC_MODEL_SUB_Y_20260615</t>
+  </si>
+  <si>
+    <t>\\sjtpo-fs.sjtpo.org\users$\Kschellinger\My Documents\ArcGIS\Projects\SJTDM_TAZ_Master\SJTDM_2020.gdb</t>
+  </si>
+  <si>
+    <t>Geodatabase</t>
+  </si>
+  <si>
+    <t>C:\Users\Kschellinger\SJTPO_Git\SJTDM_TAZ_Migration\data\derived\REC_MODEL_SUB_Y.shp</t>
   </si>
 </sst>
 </file>
@@ -2155,7 +2170,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="185.25">
+    <row r="13" spans="1:13" ht="299.25">
       <c r="A13" s="10" t="s">
         <v>226</v>
       </c>
@@ -2189,7 +2204,7 @@
       </c>
       <c r="L13" s="3"/>
       <c r="M13" s="3" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="142.5">
@@ -2226,7 +2241,7 @@
       </c>
       <c r="L14" s="3"/>
       <c r="M14" s="3" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="28.5">
@@ -6022,14 +6037,27 @@
         <v>292</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
-      <c r="A10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
+    <row r="10" spans="1:13" ht="69.75" customHeight="1">
+      <c r="A10" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="B10" t="s">
+        <v>332</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>333</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>335</v>
+      </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+      <c r="H10" s="3">
+        <v>2020</v>
+      </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>

</xml_diff>